<commit_message>
Demo workbook + apply_workbook_repairs: F7/G7 styling matches rifle-setup block
Row 7 (Turret: dropdown) styling now matches rows 5/6 (Rifle/Shooter/
Cartridge and Barrel/Optic/Chrono):

- F7 (label): horizontal=right + vertical=center alignment, yellow fill
  FFFFE082, dark blue bold font FF1F4E78, thin gray border FFB0B0B0
- G7:J7 (value merge): horizontal=left + vertical=center alignment on
  the top-left, cream fill FFFFF8E1, black font, thin gray border
  drawing the outline of the merged range
- Row 7 height bumped to 31.5 px (was 22) to match rows 5 and 6.

Turret dropdown now also includes "N/A" as a fifth option, for scopes
without an adjustable turret. List is canonical across both sheets:
"0.1 Mil, 0.05 Mil, 1/4 MOA, 1/8 MOA, N/A".

Both fixes applied in apply_workbook_repairs so real user imports also
get the consistent styling, not just the bundled demo workbook.

Tests: 114/114 passing.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/resources/Loadscope - Demo Workbook.xlsx
+++ b/app/resources/Loadscope - Demo Workbook.xlsx
@@ -52,7 +52,7 @@
     <numFmt numFmtId="180" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="181" formatCode="mm/dd/yyyy"/>
   </numFmts>
-  <fonts count="64">
+  <fonts count="66">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -455,10 +455,17 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="FF1F4E78"/>
+    </font>
+    <font>
+      <color rgb="FF000000"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="FFFFFF00"/>
     </font>
   </fonts>
-  <fills count="41">
+  <fills count="42">
     <fill>
       <patternFill/>
     </fill>
@@ -692,8 +699,14 @@
         <bgColor rgb="FFEFEFEF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE082"/>
+        <bgColor rgb="FFFFE082"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="30">
+  <borders count="31">
     <border>
       <left/>
       <right/>
@@ -983,6 +996,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB0B0B0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -994,7 +1021,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="586">
+  <cellXfs count="590">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2806,8 +2833,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="63" fillId="38" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="65" fillId="38" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="41" borderId="30" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="64" fillId="25" borderId="30" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="181" fontId="5" fillId="16" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -2821,6 +2859,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="30" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
     <xf numFmtId="2" fontId="7" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -9486,25 +9528,25 @@
       <c r="AF6" s="317" t="n"/>
       <c r="AG6" s="317" t="n"/>
     </row>
-    <row r="7" ht="22" customHeight="1" s="141">
+    <row r="7" ht="31.5" customHeight="1" s="141">
       <c r="A7" s="317" t="n"/>
       <c r="B7" s="317" t="n"/>
       <c r="C7" s="317" t="n"/>
       <c r="D7" s="317" t="n"/>
       <c r="E7" s="317" t="n"/>
-      <c r="F7" s="317" t="inlineStr">
-        <is>
-          <t>Scope click:</t>
-        </is>
-      </c>
-      <c r="G7" s="317" t="inlineStr">
+      <c r="F7" s="580" t="inlineStr">
+        <is>
+          <t>Turret:</t>
+        </is>
+      </c>
+      <c r="G7" s="581" t="inlineStr">
         <is>
           <t>0.1 Mil</t>
         </is>
       </c>
-      <c r="H7" s="309" t="n"/>
-      <c r="I7" s="309" t="n"/>
-      <c r="J7" s="309" t="n"/>
+      <c r="H7" s="582" t="n"/>
+      <c r="I7" s="582" t="n"/>
+      <c r="J7" s="582" t="n"/>
       <c r="K7" s="317" t="n"/>
       <c r="L7" s="317" t="n"/>
       <c r="M7" s="317" t="n"/>
@@ -9767,7 +9809,7 @@
           <t>Date:</t>
         </is>
       </c>
-      <c r="B13" s="580" t="n">
+      <c r="B13" s="583" t="n">
         <v>46124</v>
       </c>
       <c r="C13" s="322" t="n"/>
@@ -12070,8 +12112,8 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G7" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"0.1 Mil,0.05 Mil,1/4 MOA,1/8 MOA"</formula1>
+    <dataValidation sqref="G7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"0.1 Mil,0.05 Mil,1/4 MOA,1/8 MOA,N/A"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -12216,11 +12258,11 @@
       <c r="A4" s="309" t="n"/>
       <c r="B4" s="506" t="n"/>
       <c r="C4" s="507" t="n"/>
-      <c r="D4" s="581">
+      <c r="D4" s="584">
         <f>IF($B$100="window","Vel Spread:","")</f>
         <v/>
       </c>
-      <c r="E4" s="582">
+      <c r="E4" s="585">
         <f>IF($B$100="window",IFERROR(INDEX(D18:D25,MATCH(MIN(L18:L25),L18:L25,0)),""),"")</f>
         <v/>
       </c>
@@ -12290,17 +12332,17 @@
           <t>→  Save Suggested Load to Library  ←</t>
         </is>
       </c>
-      <c r="B6" s="583" t="n"/>
-      <c r="C6" s="583" t="n"/>
-      <c r="D6" s="583" t="n"/>
-      <c r="E6" s="583" t="n"/>
-      <c r="F6" s="583" t="n"/>
-      <c r="G6" s="583" t="n"/>
-      <c r="H6" s="583" t="n"/>
-      <c r="I6" s="583" t="n"/>
-      <c r="J6" s="583" t="n"/>
-      <c r="K6" s="583" t="n"/>
-      <c r="L6" s="584" t="n"/>
+      <c r="B6" s="586" t="n"/>
+      <c r="C6" s="586" t="n"/>
+      <c r="D6" s="586" t="n"/>
+      <c r="E6" s="586" t="n"/>
+      <c r="F6" s="586" t="n"/>
+      <c r="G6" s="586" t="n"/>
+      <c r="H6" s="586" t="n"/>
+      <c r="I6" s="586" t="n"/>
+      <c r="J6" s="586" t="n"/>
+      <c r="K6" s="586" t="n"/>
+      <c r="L6" s="587" t="n"/>
       <c r="M6" s="309" t="n"/>
       <c r="N6" s="309" t="n"/>
       <c r="O6" s="309" t="n"/>
@@ -12475,17 +12517,17 @@
           <t>→  Reset weights to Loadscope defaults  ←</t>
         </is>
       </c>
-      <c r="B12" s="583" t="n"/>
-      <c r="C12" s="583" t="n"/>
-      <c r="D12" s="583" t="n"/>
-      <c r="E12" s="583" t="n"/>
-      <c r="F12" s="583" t="n"/>
-      <c r="G12" s="583" t="n"/>
-      <c r="H12" s="583" t="n"/>
-      <c r="I12" s="583" t="n"/>
-      <c r="J12" s="583" t="n"/>
-      <c r="K12" s="583" t="n"/>
-      <c r="L12" s="584" t="n"/>
+      <c r="B12" s="586" t="n"/>
+      <c r="C12" s="586" t="n"/>
+      <c r="D12" s="586" t="n"/>
+      <c r="E12" s="586" t="n"/>
+      <c r="F12" s="586" t="n"/>
+      <c r="G12" s="586" t="n"/>
+      <c r="H12" s="586" t="n"/>
+      <c r="I12" s="586" t="n"/>
+      <c r="J12" s="586" t="n"/>
+      <c r="K12" s="586" t="n"/>
+      <c r="L12" s="587" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1" s="141">
       <c r="A13" s="349" t="inlineStr">
@@ -14828,25 +14870,25 @@
       <c r="AK6" s="317" t="n"/>
       <c r="AL6" s="317" t="n"/>
     </row>
-    <row r="7" ht="22" customHeight="1" s="141">
+    <row r="7" ht="31.5" customHeight="1" s="141">
       <c r="A7" s="317" t="n"/>
       <c r="B7" s="317" t="n"/>
       <c r="C7" s="317" t="n"/>
       <c r="D7" s="317" t="n"/>
       <c r="E7" s="317" t="n"/>
-      <c r="F7" s="317" t="inlineStr">
-        <is>
-          <t>Scope click:</t>
-        </is>
-      </c>
-      <c r="G7" s="317" t="inlineStr">
+      <c r="F7" s="580" t="inlineStr">
+        <is>
+          <t>Turret:</t>
+        </is>
+      </c>
+      <c r="G7" s="581" t="inlineStr">
         <is>
           <t>0.1 Mil</t>
         </is>
       </c>
-      <c r="H7" s="317" t="n"/>
-      <c r="I7" s="317" t="n"/>
-      <c r="J7" s="317" t="n"/>
+      <c r="H7" s="588" t="n"/>
+      <c r="I7" s="588" t="n"/>
+      <c r="J7" s="588" t="n"/>
       <c r="K7" s="317" t="n"/>
       <c r="L7" s="317" t="n"/>
       <c r="M7" s="317" t="n"/>
@@ -15139,7 +15181,7 @@
           <t>Date:</t>
         </is>
       </c>
-      <c r="B13" s="580" t="n">
+      <c r="B13" s="583" t="n">
         <v>46138</v>
       </c>
       <c r="C13" s="322" t="n"/>
@@ -16208,21 +16250,21 @@
           <t>→  Save Suggested Load to Library  ←</t>
         </is>
       </c>
-      <c r="B26" s="583" t="n"/>
-      <c r="C26" s="583" t="n"/>
-      <c r="D26" s="583" t="n"/>
-      <c r="E26" s="583" t="n"/>
-      <c r="F26" s="583" t="n"/>
-      <c r="G26" s="583" t="n"/>
-      <c r="H26" s="583" t="n"/>
-      <c r="I26" s="583" t="n"/>
-      <c r="J26" s="583" t="n"/>
-      <c r="K26" s="583" t="n"/>
-      <c r="L26" s="583" t="n"/>
-      <c r="M26" s="583" t="n"/>
-      <c r="N26" s="583" t="n"/>
-      <c r="O26" s="583" t="n"/>
-      <c r="P26" s="584" t="n"/>
+      <c r="B26" s="586" t="n"/>
+      <c r="C26" s="586" t="n"/>
+      <c r="D26" s="586" t="n"/>
+      <c r="E26" s="586" t="n"/>
+      <c r="F26" s="586" t="n"/>
+      <c r="G26" s="586" t="n"/>
+      <c r="H26" s="586" t="n"/>
+      <c r="I26" s="586" t="n"/>
+      <c r="J26" s="586" t="n"/>
+      <c r="K26" s="586" t="n"/>
+      <c r="L26" s="586" t="n"/>
+      <c r="M26" s="586" t="n"/>
+      <c r="N26" s="586" t="n"/>
+      <c r="O26" s="586" t="n"/>
+      <c r="P26" s="587" t="n"/>
       <c r="Q26" s="317" t="n"/>
       <c r="R26" s="317" t="n"/>
       <c r="S26" s="317" t="n"/>
@@ -16291,7 +16333,7 @@
       <c r="AL27" s="317" t="n"/>
     </row>
     <row r="28" ht="32" customHeight="1" s="141">
-      <c r="A28" s="585" t="inlineStr">
+      <c r="A28" s="589" t="inlineStr">
         <is>
           <t>→  Reset weights (hover for rationale)  ←</t>
         </is>
@@ -19532,7 +19574,7 @@
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="G7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"0.1 Mil,0.05 Mil,1/4 MOA,1/8 MOA"</formula1>
+      <formula1>"0.1 Mil,0.05 Mil,1/4 MOA,1/8 MOA,N/A"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -25826,16 +25868,16 @@
           <t>→  Print Pocket Range Card  ←</t>
         </is>
       </c>
-      <c r="B2" s="583" t="n"/>
-      <c r="C2" s="583" t="n"/>
-      <c r="D2" s="583" t="n"/>
-      <c r="E2" s="583" t="n"/>
-      <c r="F2" s="583" t="n"/>
-      <c r="G2" s="583" t="n"/>
-      <c r="H2" s="583" t="n"/>
-      <c r="I2" s="583" t="n"/>
-      <c r="J2" s="583" t="n"/>
-      <c r="K2" s="584" t="n"/>
+      <c r="B2" s="586" t="n"/>
+      <c r="C2" s="586" t="n"/>
+      <c r="D2" s="586" t="n"/>
+      <c r="E2" s="586" t="n"/>
+      <c r="F2" s="586" t="n"/>
+      <c r="G2" s="586" t="n"/>
+      <c r="H2" s="586" t="n"/>
+      <c r="I2" s="586" t="n"/>
+      <c r="J2" s="586" t="n"/>
+      <c r="K2" s="587" t="n"/>
     </row>
     <row r="3" ht="6" customHeight="1" s="141">
       <c r="A3" s="309" t="n"/>
@@ -25856,16 +25898,16 @@
           <t>Enter your DOPE values in MILS or MOA. Click counts auto-calculate based on your scope's click value (set on the Load Log tab — Click: dropdown).</t>
         </is>
       </c>
-      <c r="B4" s="583" t="n"/>
-      <c r="C4" s="583" t="n"/>
-      <c r="D4" s="583" t="n"/>
-      <c r="E4" s="583" t="n"/>
-      <c r="F4" s="583" t="n"/>
-      <c r="G4" s="583" t="n"/>
-      <c r="H4" s="583" t="n"/>
-      <c r="I4" s="583" t="n"/>
-      <c r="J4" s="583" t="n"/>
-      <c r="K4" s="584" t="n"/>
+      <c r="B4" s="586" t="n"/>
+      <c r="C4" s="586" t="n"/>
+      <c r="D4" s="586" t="n"/>
+      <c r="E4" s="586" t="n"/>
+      <c r="F4" s="586" t="n"/>
+      <c r="G4" s="586" t="n"/>
+      <c r="H4" s="586" t="n"/>
+      <c r="I4" s="586" t="n"/>
+      <c r="J4" s="586" t="n"/>
+      <c r="K4" s="587" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1" s="141">
       <c r="A5" s="381" t="inlineStr">

</xml_diff>

<commit_message>
Demo workbook: Load Library readable widths + wrapped notes
Six column widths bumped on Load Library so the demo entries are
readable without column-resize gymnastics:
- E (Bullet): default -> 18
- G (Powder): 9 -> 16 ("Hodgdon H4350" needed room)
- J (Brass): default -> 12
- M (Avg Vel): default -> 12
- P (MR MOA): default -> 10
- Q (Notes/Conditions): 12 -> 28 + wrap_text on data rows + row height 32

Page orientation was already landscape from the template - no change.

Pocket Range Card preview placement on Ballistics tab is deferred to a
later iteration (the existing "Print Pocket Range Card" button at A2
already opens the rendered card in the user's browser - the duplicate
in-Excel preview would be meaningful additional design work).

Tests: 114/114 passing.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/resources/Loadscope - Demo Workbook.xlsx
+++ b/app/resources/Loadscope - Demo Workbook.xlsx
@@ -1021,7 +1021,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="592">
+  <cellXfs count="594">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2869,8 +2869,16 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
     <xf numFmtId="181" fontId="14" fillId="3" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
@@ -25069,15 +25077,19 @@
     <col width="12" customWidth="1" style="140" min="2" max="2"/>
     <col width="36" customWidth="1" style="140" min="3" max="3"/>
     <col width="22" customWidth="1" style="140" min="4" max="5"/>
+    <col width="18" customWidth="1" style="141" min="5" max="5"/>
     <col width="11" customWidth="1" style="140" min="6" max="6"/>
-    <col width="9" customWidth="1" style="140" min="7" max="7"/>
+    <col width="16" customWidth="1" style="140" min="7" max="7"/>
     <col width="11" customWidth="1" style="140" min="8" max="8"/>
     <col width="12" customWidth="1" style="140" min="9" max="10"/>
+    <col width="12" customWidth="1" style="141" min="10" max="10"/>
     <col width="22" customWidth="1" style="140" min="11" max="11"/>
     <col width="11" customWidth="1" style="140" min="12" max="13"/>
+    <col width="12" customWidth="1" style="141" min="13" max="13"/>
     <col width="12" customWidth="1" style="140" min="14" max="14"/>
     <col width="9" customWidth="1" style="140" min="15" max="16"/>
-    <col width="12" customWidth="1" style="140" min="17" max="17"/>
+    <col width="10" customWidth="1" style="141" min="16" max="16"/>
+    <col width="28" customWidth="1" style="140" min="17" max="17"/>
     <col width="8.43" customWidth="1" style="140" min="18" max="29"/>
   </cols>
   <sheetData>
@@ -25285,7 +25297,7 @@
       <c r="Y4" s="317" t="n"/>
       <c r="Z4" s="317" t="n"/>
     </row>
-    <row r="5" ht="21.75" customHeight="1" s="141">
+    <row r="5" ht="32" customHeight="1" s="141">
       <c r="A5" s="359" t="n">
         <v>1</v>
       </c>
@@ -25346,7 +25358,7 @@
       <c r="P5" s="376" t="n">
         <v>0.18</v>
       </c>
-      <c r="Q5" s="359" t="inlineStr">
+      <c r="Q5" s="591" t="inlineStr">
         <is>
           <t>Confirmed at 100 yd, 65°F, 1500 ft DA. 10-shot string.</t>
         </is>
@@ -25361,11 +25373,11 @@
       <c r="Y5" s="317" t="n"/>
       <c r="Z5" s="317" t="n"/>
     </row>
-    <row r="6" ht="21.75" customHeight="1" s="141">
+    <row r="6" ht="32" customHeight="1" s="141">
       <c r="A6" s="336" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="591" t="n">
+      <c r="B6" s="592" t="n">
         <v>45971</v>
       </c>
       <c r="C6" s="336" t="inlineStr">
@@ -25422,7 +25434,7 @@
       <c r="P6" s="380" t="n">
         <v>0.24</v>
       </c>
-      <c r="Q6" s="336" t="inlineStr">
+      <c r="Q6" s="593" t="inlineStr">
         <is>
           <t>Prior season — switched to ELD-M for lower SD.</t>
         </is>
@@ -25437,7 +25449,7 @@
       <c r="Y6" s="317" t="n"/>
       <c r="Z6" s="317" t="n"/>
     </row>
-    <row r="7" ht="21.75" customHeight="1" s="141">
+    <row r="7" ht="32" customHeight="1" s="141">
       <c r="A7" s="359" t="n">
         <v>3</v>
       </c>
@@ -25498,7 +25510,7 @@
       <c r="P7" s="376" t="n">
         <v>0.28</v>
       </c>
-      <c r="Q7" s="359" t="inlineStr">
+      <c r="Q7" s="591" t="inlineStr">
         <is>
           <t>Truck gun build. Good cold-bore consistency.</t>
         </is>

</xml_diff>

<commit_message>
Range Card tab: visual overhaul to look like a printed card, not a spreadsheet
Per Chad's feedback ("can it look more like the card is going to look?"),
the Range Card tab now mirrors the polished HTML print version aesthetic:

- Hidden Excel gridlines (sheet_view.showGridLines = False)
- Hidden row/column headers
- Zoom set to 125% so the card fills the viewport on open
- Helvetica Neue typography (matches the HTML card)
- Title row: 22pt bold dark blue + bottom underline (instead of solid color bar)
- Subtitle (rifle/bullet/charge/vel): 13pt bold dark blue on white (instead
  of yellow fill)
- Scope info: 11pt subtle gray
- DOPE table: dark blue header band + subtle alternating row stripes
  (F7F9FC light blue-gray) for readability
- Padding rows between sections for breathing room
- Footer: muted gray italic note pointing to the Print button

Tests: 114/114 passing.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/resources/Loadscope - Demo Workbook.xlsx
+++ b/app/resources/Loadscope - Demo Workbook.xlsx
@@ -53,7 +53,7 @@
     <numFmt numFmtId="180" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="181" formatCode="mm/dd/yyyy"/>
   </numFmts>
-  <fonts count="71">
+  <fonts count="72">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -466,31 +466,41 @@
       <color rgb="FFFFFF00"/>
     </font>
     <font>
+      <name val="Helvetica Neue"/>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="16"/>
+      <color rgb="FF1F4E78"/>
+      <sz val="22"/>
     </font>
     <font>
+      <name val="Helvetica Neue"/>
       <b val="1"/>
       <color rgb="FF1F4E78"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Helvetica Neue"/>
+      <color rgb="FF555555"/>
       <sz val="11"/>
     </font>
     <font>
-      <i val="1"/>
-      <color rgb="FF555555"/>
-      <sz val="10"/>
-    </font>
-    <font>
+      <name val="Helvetica Neue"/>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
+      <name val="Helvetica Neue"/>
       <color rgb="FF000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Helvetica Neue"/>
+      <i val="1"/>
+      <color rgb="FF888888"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="42">
+  <fills count="44">
     <fill>
       <patternFill/>
     </fill>
@@ -730,8 +740,20 @@
         <bgColor rgb="FFFFE082"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF7F9FC"/>
+        <bgColor rgb="FFF7F9FC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="32">
+  <borders count="33">
     <border>
       <left/>
       <right/>
@@ -1036,17 +1058,22 @@
       </bottom>
     </border>
     <border>
+      <bottom style="medium">
+        <color rgb="FF1F4E78"/>
+      </bottom>
+    </border>
+    <border>
       <left style="thin">
-        <color rgb="FF888888"/>
+        <color rgb="FFBBBBBB"/>
       </left>
       <right style="thin">
-        <color rgb="FF888888"/>
+        <color rgb="FFBBBBBB"/>
       </right>
       <top style="thin">
-        <color rgb="FF888888"/>
+        <color rgb="FFBBBBBB"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF888888"/>
+        <color rgb="FFBBBBBB"/>
       </bottom>
     </border>
   </borders>
@@ -1060,7 +1087,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="600">
+  <cellXfs count="603">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2920,22 +2947,27 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="66" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="66" fillId="42" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="67" fillId="41" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="67" fillId="42" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="68" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="68" fillId="42" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="69" fillId="26" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="42" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="69" fillId="21" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="70" fillId="0" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="70" fillId="42" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="68" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="70" fillId="43" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="42" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -29346,423 +29378,456 @@
   <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" style="141" min="1" max="1"/>
+    <col width="11" customWidth="1" style="141" min="1" max="1"/>
     <col width="8" customWidth="1" style="141" min="2" max="2"/>
     <col width="8" customWidth="1" style="141" min="3" max="3"/>
     <col width="8" customWidth="1" style="141" min="4" max="4"/>
     <col width="8" customWidth="1" style="141" min="5" max="5"/>
-    <col width="8" customWidth="1" style="141" min="6" max="6"/>
+    <col width="9" customWidth="1" style="141" min="6" max="6"/>
     <col width="8" customWidth="1" style="141" min="7" max="7"/>
-    <col width="8" customWidth="1" style="141" min="8" max="8"/>
+    <col width="9" customWidth="1" style="141" min="8" max="8"/>
     <col width="8" customWidth="1" style="141" min="9" max="9"/>
-    <col width="8" customWidth="1" style="141" min="10" max="10"/>
+    <col width="9" customWidth="1" style="141" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" s="141">
+    <row r="1" ht="36" customHeight="1" s="141">
       <c r="A1" s="594" t="inlineStr">
         <is>
           <t>POCKET RANGE CARD</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="22" customHeight="1" s="141">
-      <c r="A2" s="595" t="inlineStr">
+      <c r="B1" s="595" t="n"/>
+      <c r="C1" s="595" t="n"/>
+      <c r="D1" s="595" t="n"/>
+      <c r="E1" s="595" t="n"/>
+      <c r="F1" s="595" t="n"/>
+      <c r="G1" s="595" t="n"/>
+      <c r="H1" s="595" t="n"/>
+      <c r="I1" s="595" t="n"/>
+      <c r="J1" s="595" t="n"/>
+    </row>
+    <row r="2" ht="26" customHeight="1" s="141">
+      <c r="A2" s="596" t="inlineStr">
         <is>
           <t>Tikka T3X CTR 6.5 CM  •  Hornady 140gr ELD-M  •  42.4gr  •  2780 fps</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="18" customHeight="1" s="141">
-      <c r="A3" s="596" t="inlineStr">
-        <is>
-          <t>Scope: Leupold Mark 5HD 5-25x56   |   Click: 0.1 Mil   |   Zero: 100 yd   |   Sight Ht: 1.75"   |   Twist: 1:8 RH</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1" s="141">
-      <c r="A5" s="597" t="inlineStr">
+    <row r="3" ht="22" customHeight="1" s="141">
+      <c r="A3" s="597" t="inlineStr">
+        <is>
+          <t>Scope: Leupold Mark 5HD 5-25x56   ·   Click: 0.1 Mil   ·   Zero: 100 yd   ·   Sight Ht: 1.75"   ·   Twist: 1:8 RH</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="8" customHeight="1" s="141">
+      <c r="A4" s="598" t="n"/>
+      <c r="B4" s="598" t="n"/>
+      <c r="C4" s="598" t="n"/>
+      <c r="D4" s="598" t="n"/>
+      <c r="E4" s="598" t="n"/>
+      <c r="F4" s="598" t="n"/>
+      <c r="G4" s="598" t="n"/>
+      <c r="H4" s="598" t="n"/>
+      <c r="I4" s="598" t="n"/>
+      <c r="J4" s="598" t="n"/>
+    </row>
+    <row r="5" ht="34" customHeight="1" s="141">
+      <c r="A5" s="599" t="inlineStr">
         <is>
           <t>Range
 (yd)</t>
         </is>
       </c>
-      <c r="B5" s="597" t="inlineStr">
+      <c r="B5" s="599" t="inlineStr">
         <is>
           <t>Mils
 Elev</t>
         </is>
       </c>
-      <c r="C5" s="597" t="inlineStr">
+      <c r="C5" s="599" t="inlineStr">
         <is>
           <t>Mil
 Clicks</t>
         </is>
       </c>
-      <c r="D5" s="597" t="inlineStr">
+      <c r="D5" s="599" t="inlineStr">
         <is>
           <t>MOA
 Elev</t>
         </is>
       </c>
-      <c r="E5" s="597" t="inlineStr">
+      <c r="E5" s="599" t="inlineStr">
         <is>
           <t>MOA
 Clicks</t>
         </is>
       </c>
-      <c r="F5" s="597" t="inlineStr">
+      <c r="F5" s="599" t="inlineStr">
         <is>
           <t>Wind
 Mils/10</t>
         </is>
       </c>
-      <c r="G5" s="597" t="inlineStr">
+      <c r="G5" s="599" t="inlineStr">
         <is>
           <t>Wind
 Mil Clk</t>
         </is>
       </c>
-      <c r="H5" s="597" t="inlineStr">
+      <c r="H5" s="599" t="inlineStr">
         <is>
           <t>Wind
 MOA/10</t>
         </is>
       </c>
-      <c r="I5" s="597" t="inlineStr">
+      <c r="I5" s="599" t="inlineStr">
         <is>
           <t>Wind
 MOA Clk</t>
         </is>
       </c>
-      <c r="J5" s="597" t="inlineStr">
+      <c r="J5" s="599" t="inlineStr">
         <is>
           <t>TOF
 (sec)</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1" s="141">
-      <c r="A6" s="598" t="n">
+    <row r="6" ht="20" customHeight="1" s="141">
+      <c r="A6" s="600" t="n">
         <v>100</v>
       </c>
-      <c r="B6" s="598" t="n">
+      <c r="B6" s="600" t="n">
         <v>0</v>
       </c>
-      <c r="C6" s="598" t="n">
+      <c r="C6" s="600" t="n">
         <v>0</v>
       </c>
-      <c r="D6" s="598" t="n">
+      <c r="D6" s="600" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="598" t="n">
+      <c r="E6" s="600" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="598" t="n">
+      <c r="F6" s="600" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="598" t="n">
+      <c r="G6" s="600" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="598" t="n">
+      <c r="H6" s="600" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="598" t="n">
+      <c r="I6" s="600" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="598" t="n">
+      <c r="J6" s="600" t="n">
         <v>0.11</v>
       </c>
     </row>
-    <row r="7" ht="18" customHeight="1" s="141">
-      <c r="A7" s="598" t="n">
+    <row r="7" ht="20" customHeight="1" s="141">
+      <c r="A7" s="601" t="n">
         <v>200</v>
       </c>
-      <c r="B7" s="598" t="n">
+      <c r="B7" s="601" t="n">
         <v>0.1</v>
       </c>
-      <c r="C7" s="598" t="n">
+      <c r="C7" s="601" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="598" t="n">
+      <c r="D7" s="601" t="n">
         <v>0.5</v>
       </c>
-      <c r="E7" s="598" t="n">
+      <c r="E7" s="601" t="n">
         <v>2</v>
       </c>
-      <c r="F7" s="598" t="n">
+      <c r="F7" s="601" t="n">
         <v>0.3</v>
       </c>
-      <c r="G7" s="598" t="n">
+      <c r="G7" s="601" t="n">
         <v>3</v>
       </c>
-      <c r="H7" s="598" t="n">
+      <c r="H7" s="601" t="n">
         <v>1</v>
       </c>
-      <c r="I7" s="598" t="n">
+      <c r="I7" s="601" t="n">
         <v>4</v>
       </c>
-      <c r="J7" s="598" t="n">
+      <c r="J7" s="601" t="n">
         <v>0.23</v>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1" s="141">
-      <c r="A8" s="598" t="n">
+    <row r="8" ht="20" customHeight="1" s="141">
+      <c r="A8" s="600" t="n">
         <v>300</v>
       </c>
-      <c r="B8" s="598" t="n">
+      <c r="B8" s="600" t="n">
         <v>0.6</v>
       </c>
-      <c r="C8" s="598" t="n">
+      <c r="C8" s="600" t="n">
         <v>6</v>
       </c>
-      <c r="D8" s="598" t="n">
+      <c r="D8" s="600" t="n">
         <v>2</v>
       </c>
-      <c r="E8" s="598" t="n">
+      <c r="E8" s="600" t="n">
         <v>8</v>
       </c>
-      <c r="F8" s="598" t="n">
+      <c r="F8" s="600" t="n">
         <v>0.5</v>
       </c>
-      <c r="G8" s="598" t="n">
+      <c r="G8" s="600" t="n">
         <v>5</v>
       </c>
-      <c r="H8" s="598" t="n">
+      <c r="H8" s="600" t="n">
         <v>1.7</v>
       </c>
-      <c r="I8" s="598" t="n">
+      <c r="I8" s="600" t="n">
         <v>7</v>
       </c>
-      <c r="J8" s="598" t="n">
+      <c r="J8" s="600" t="n">
         <v>0.36</v>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1" s="141">
-      <c r="A9" s="598" t="n">
+    <row r="9" ht="20" customHeight="1" s="141">
+      <c r="A9" s="601" t="n">
         <v>400</v>
       </c>
-      <c r="B9" s="598" t="n">
+      <c r="B9" s="601" t="n">
         <v>1.2</v>
       </c>
-      <c r="C9" s="598" t="n">
+      <c r="C9" s="601" t="n">
         <v>12</v>
       </c>
-      <c r="D9" s="598" t="n">
+      <c r="D9" s="601" t="n">
         <v>4.1</v>
       </c>
-      <c r="E9" s="598" t="n">
+      <c r="E9" s="601" t="n">
         <v>16</v>
       </c>
-      <c r="F9" s="598" t="n">
+      <c r="F9" s="601" t="n">
         <v>0.7</v>
       </c>
-      <c r="G9" s="598" t="n">
+      <c r="G9" s="601" t="n">
         <v>7</v>
       </c>
-      <c r="H9" s="598" t="n">
+      <c r="H9" s="601" t="n">
         <v>2.4</v>
       </c>
-      <c r="I9" s="598" t="n">
+      <c r="I9" s="601" t="n">
         <v>10</v>
       </c>
-      <c r="J9" s="598" t="n">
+      <c r="J9" s="601" t="n">
         <v>0.5</v>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1" s="141">
-      <c r="A10" s="598" t="n">
+    <row r="10" ht="20" customHeight="1" s="141">
+      <c r="A10" s="600" t="n">
         <v>500</v>
       </c>
-      <c r="B10" s="598" t="n">
+      <c r="B10" s="600" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="598" t="n">
+      <c r="C10" s="600" t="n">
         <v>20</v>
       </c>
-      <c r="D10" s="598" t="n">
+      <c r="D10" s="600" t="n">
         <v>6.9</v>
       </c>
-      <c r="E10" s="598" t="n">
+      <c r="E10" s="600" t="n">
         <v>28</v>
       </c>
-      <c r="F10" s="598" t="n">
+      <c r="F10" s="600" t="n">
         <v>0.9</v>
       </c>
-      <c r="G10" s="598" t="n">
+      <c r="G10" s="600" t="n">
         <v>9</v>
       </c>
-      <c r="H10" s="598" t="n">
+      <c r="H10" s="600" t="n">
         <v>3.1</v>
       </c>
-      <c r="I10" s="598" t="n">
+      <c r="I10" s="600" t="n">
         <v>12</v>
       </c>
-      <c r="J10" s="598" t="n">
+      <c r="J10" s="600" t="n">
         <v>0.66</v>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1" s="141">
-      <c r="A11" s="598" t="n">
+    <row r="11" ht="20" customHeight="1" s="141">
+      <c r="A11" s="601" t="n">
         <v>600</v>
       </c>
-      <c r="B11" s="598" t="n">
+      <c r="B11" s="601" t="n">
         <v>2.8</v>
       </c>
-      <c r="C11" s="598" t="n">
+      <c r="C11" s="601" t="n">
         <v>28</v>
       </c>
-      <c r="D11" s="598" t="n">
+      <c r="D11" s="601" t="n">
         <v>9.6</v>
       </c>
-      <c r="E11" s="598" t="n">
+      <c r="E11" s="601" t="n">
         <v>38</v>
       </c>
-      <c r="F11" s="598" t="n">
+      <c r="F11" s="601" t="n">
         <v>1.2</v>
       </c>
-      <c r="G11" s="598" t="n">
+      <c r="G11" s="601" t="n">
         <v>12</v>
       </c>
-      <c r="H11" s="598" t="n">
+      <c r="H11" s="601" t="n">
         <v>4.1</v>
       </c>
-      <c r="I11" s="598" t="n">
+      <c r="I11" s="601" t="n">
         <v>16</v>
       </c>
-      <c r="J11" s="598" t="n">
+      <c r="J11" s="601" t="n">
         <v>0.83</v>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1" s="141">
-      <c r="A12" s="598" t="n">
+    <row r="12" ht="20" customHeight="1" s="141">
+      <c r="A12" s="600" t="n">
         <v>700</v>
       </c>
-      <c r="B12" s="598" t="n">
+      <c r="B12" s="600" t="n">
         <v>3.7</v>
       </c>
-      <c r="C12" s="598" t="n">
+      <c r="C12" s="600" t="n">
         <v>37</v>
       </c>
-      <c r="D12" s="598" t="n">
+      <c r="D12" s="600" t="n">
         <v>12.7</v>
       </c>
-      <c r="E12" s="598" t="n">
+      <c r="E12" s="600" t="n">
         <v>51</v>
       </c>
-      <c r="F12" s="598" t="n">
+      <c r="F12" s="600" t="n">
         <v>1.5</v>
       </c>
-      <c r="G12" s="598" t="n">
+      <c r="G12" s="600" t="n">
         <v>15</v>
       </c>
-      <c r="H12" s="598" t="n">
+      <c r="H12" s="600" t="n">
         <v>5.1</v>
       </c>
-      <c r="I12" s="598" t="n">
+      <c r="I12" s="600" t="n">
         <v>20</v>
       </c>
-      <c r="J12" s="598" t="n">
+      <c r="J12" s="600" t="n">
         <v>1.02</v>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1" s="141">
-      <c r="A13" s="598" t="n">
+    <row r="13" ht="20" customHeight="1" s="141">
+      <c r="A13" s="601" t="n">
         <v>800</v>
       </c>
-      <c r="B13" s="598" t="n">
+      <c r="B13" s="601" t="n">
         <v>4.8</v>
       </c>
-      <c r="C13" s="598" t="n">
+      <c r="C13" s="601" t="n">
         <v>48</v>
       </c>
-      <c r="D13" s="598" t="n">
+      <c r="D13" s="601" t="n">
         <v>16.5</v>
       </c>
-      <c r="E13" s="598" t="n">
+      <c r="E13" s="601" t="n">
         <v>66</v>
       </c>
-      <c r="F13" s="598" t="n">
+      <c r="F13" s="601" t="n">
         <v>1.8</v>
       </c>
-      <c r="G13" s="598" t="n">
+      <c r="G13" s="601" t="n">
         <v>18</v>
       </c>
-      <c r="H13" s="598" t="n">
+      <c r="H13" s="601" t="n">
         <v>6.2</v>
       </c>
-      <c r="I13" s="598" t="n">
+      <c r="I13" s="601" t="n">
         <v>25</v>
       </c>
-      <c r="J13" s="598" t="n">
+      <c r="J13" s="601" t="n">
         <v>1.23</v>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1" s="141">
-      <c r="A14" s="598" t="n">
+    <row r="14" ht="20" customHeight="1" s="141">
+      <c r="A14" s="600" t="n">
         <v>900</v>
       </c>
-      <c r="B14" s="598" t="n">
+      <c r="B14" s="600" t="n">
         <v>6</v>
       </c>
-      <c r="C14" s="598" t="n">
+      <c r="C14" s="600" t="n">
         <v>60</v>
       </c>
-      <c r="D14" s="598" t="n">
+      <c r="D14" s="600" t="n">
         <v>20.6</v>
       </c>
-      <c r="E14" s="598" t="n">
+      <c r="E14" s="600" t="n">
         <v>82</v>
       </c>
-      <c r="F14" s="598" t="n">
+      <c r="F14" s="600" t="n">
         <v>2.1</v>
       </c>
-      <c r="G14" s="598" t="n">
+      <c r="G14" s="600" t="n">
         <v>21</v>
       </c>
-      <c r="H14" s="598" t="n">
+      <c r="H14" s="600" t="n">
         <v>7.2</v>
       </c>
-      <c r="I14" s="598" t="n">
+      <c r="I14" s="600" t="n">
         <v>29</v>
       </c>
-      <c r="J14" s="598" t="n">
+      <c r="J14" s="600" t="n">
         <v>1.46</v>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1" s="141">
-      <c r="A15" s="598" t="n">
+    <row r="15" ht="20" customHeight="1" s="141">
+      <c r="A15" s="601" t="n">
         <v>1000</v>
       </c>
-      <c r="B15" s="598" t="n">
+      <c r="B15" s="601" t="n">
         <v>7.3</v>
       </c>
-      <c r="C15" s="598" t="n">
+      <c r="C15" s="601" t="n">
         <v>73</v>
       </c>
-      <c r="D15" s="598" t="n">
+      <c r="D15" s="601" t="n">
         <v>25</v>
       </c>
-      <c r="E15" s="598" t="n">
+      <c r="E15" s="601" t="n">
         <v>100</v>
       </c>
-      <c r="F15" s="598" t="n">
+      <c r="F15" s="601" t="n">
         <v>2.4</v>
       </c>
-      <c r="G15" s="598" t="n">
+      <c r="G15" s="601" t="n">
         <v>24</v>
       </c>
-      <c r="H15" s="598" t="n">
+      <c r="H15" s="601" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="I15" s="598" t="n">
+      <c r="I15" s="601" t="n">
         <v>33</v>
       </c>
-      <c r="J15" s="598" t="n">
+      <c r="J15" s="601" t="n">
         <v>1.71</v>
       </c>
     </row>
-    <row r="17" ht="36" customHeight="1" s="141">
-      <c r="A17" s="599" t="inlineStr">
+    <row r="16" ht="8" customHeight="1" s="141">
+      <c r="A16" s="598" t="n"/>
+      <c r="B16" s="598" t="n"/>
+      <c r="C16" s="598" t="n"/>
+      <c r="D16" s="598" t="n"/>
+      <c r="E16" s="598" t="n"/>
+      <c r="F16" s="598" t="n"/>
+      <c r="G16" s="598" t="n"/>
+      <c r="H16" s="598" t="n"/>
+      <c r="I16" s="598" t="n"/>
+      <c r="J16" s="598" t="n"/>
+    </row>
+    <row r="17" ht="32" customHeight="1" s="141">
+      <c r="A17" s="602" t="inlineStr">
         <is>
           <t>Click "Print Pocket Range Card" on the Ballistics tab to print this card as a 4×6 page.</t>
         </is>

</xml_diff>

<commit_message>
Ballistics row 5/6: merge B:C so long rifle/scope names fit
apply_workbook_repairs now merges Ballistics!B5:C5 and B6:C6 so long
rifle and scope names (e.g., "Leupold Mark 5HD 5-25x56" at 24 chars)
fit without being clipped by the default col B width of 13. Also
disables wrap_text on those cells so the name stays on a single line
in the merged 26-char width.

Doesn't disturb the DOPE table below (rows 9-18) - those rows are
unaffected by row 5/6 merges.

Affects real user imports too since the same merge is added on every
import via apply_workbook_repairs.

Tests: 114/114 passing.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/resources/Loadscope - Demo Workbook.xlsx
+++ b/app/resources/Loadscope - Demo Workbook.xlsx
@@ -1021,7 +1021,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="594">
+  <cellXfs count="596">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2879,6 +2879,13 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
@@ -26011,12 +26018,12 @@
           <t>Rifle:</t>
         </is>
       </c>
-      <c r="B5" s="270" t="inlineStr">
+      <c r="B5" s="594" t="inlineStr">
         <is>
           <t>Tikka T3X CTR 6.5 CM</t>
         </is>
       </c>
-      <c r="C5" s="382" t="n"/>
+      <c r="C5" s="166" t="n"/>
       <c r="D5" s="381" t="inlineStr">
         <is>
           <t>Bullet:</t>
@@ -26052,12 +26059,12 @@
           <t>Scope:</t>
         </is>
       </c>
-      <c r="B6" s="363" t="inlineStr">
+      <c r="B6" s="595" t="inlineStr">
         <is>
           <t>Leupold Mark 5HD 5-25x56</t>
         </is>
       </c>
-      <c r="C6" s="384" t="n"/>
+      <c r="C6" s="323" t="n"/>
       <c r="D6" s="383" t="inlineStr">
         <is>
           <t>Zero (yd):</t>
@@ -28382,10 +28389,12 @@
     <row r="91" ht="12" customHeight="1" s="141"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="0"/>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="A58:K58"/>
     <mergeCell ref="A22:K22"/>
+    <mergeCell ref="B6:C6"/>
     <mergeCell ref="A4:K4"/>
+    <mergeCell ref="B5:C5"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A76:K76"/>
     <mergeCell ref="A1:K1"/>

</xml_diff>